<commit_message>
update visualisation + add rugby dataset
</commit_message>
<xml_diff>
--- a/data/demo_data/cardiovascular/cardio_map.xlsx
+++ b/data/demo_data/cardiovascular/cardio_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\demo_data\cardiovascular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BC986D-354B-4077-9A2D-433DC241F2AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144EB73A-5E97-46E4-82F6-FD23A77E4D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1ED84D23-49D9-4C3A-9022-4B7CCB101240}"/>
+    <workbookView xWindow="56280" yWindow="2430" windowWidth="19875" windowHeight="15225" xr2:uid="{1ED84D23-49D9-4C3A-9022-4B7CCB101240}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Key</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Value</t>
   </si>
   <si>
-    <t>id</t>
-  </si>
-  <si>
     <t>age</t>
   </si>
   <si>
@@ -84,9 +81,6 @@
     <t>cardio</t>
   </si>
   <si>
-    <t>genger</t>
-  </si>
-  <si>
     <t>Systolic blood pressure</t>
   </si>
   <si>
@@ -106,6 +100,18 @@
   </si>
   <si>
     <t>presence or absence of cardiovascular disease</t>
+  </si>
+  <si>
+    <t>age of the patient</t>
+  </si>
+  <si>
+    <t>genger of the patient</t>
+  </si>
+  <si>
+    <t>height of the patient</t>
+  </si>
+  <si>
+    <t>weight of the patient</t>
   </si>
 </sst>
 </file>
@@ -466,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D297FE0-BB8E-4B17-800B-691B6EC5BDCB}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="47.6328125" customWidth="1"/>
@@ -485,7 +491,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -493,7 +499,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -501,7 +507,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -509,7 +515,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -517,7 +523,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -525,7 +531,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -533,7 +539,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -541,7 +547,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -549,7 +555,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -557,7 +563,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -565,7 +571,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -573,15 +579,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>